<commit_message>
Fix generic filler descriptions in Units 11-12 coding questions
Same fix as prior units: rewrote the 10 placeholder descriptions in
each unit with a real scenario and explicit logic, verified against
existing solutions/test cases.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/Coding Questions/Unit 11 - File Handling/Unit 11 - File Handling - Coding Questions.xlsx
+++ b/content/Question Bank/Coding Questions/Unit 11 - File Handling/Unit 11 - File Handling - Coding Questions.xlsx
@@ -1904,17 +1904,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Line Counter. Read the input values and print the required result exactly.
+          <t>A batch import tool is told upfront how many rows a data file contains, then reads through every row one by one to make sure none are missing, and finally confirms the total number of rows it processed.
+Write a program that reads a whole number N, then reads N more lines (treat them as the file's contents, one row per line), and prints N once all the lines have been read.
 ### Input Format
-- Line 1: N
-- Next N lines: Text
+- Line 1: N, the number of lines in the file
+- Next N lines: the file's contents
 ### Output Format
 ```
 3
 ```
+### Example Walkthrough
+In the sample, N is 3 and the file contains the lines `a`, `b`, and `c`. After reading all three lines, the program prints the total, `3`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- N is a valid whole number matching the number of lines that follow.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -2076,17 +2079,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Longest File Line. Read the input values and print the required result exactly.
+          <t>A log-file linter checks the length of every line in a file to catch the single longest one, since lines over a certain length must be flagged for readability.
+Write a program that reads a whole number N, then reads N more lines (treat them as the file's contents), and prints the length of the longest line. If N is 0, print `0`.
 ### Input Format
-- Line 1: N
-- Next N lines: Text
+- Line 1: N, the number of lines in the file
+- Next N lines: the file's contents
 ### Output Format
 ```
 3
 ```
+### Example Walkthrough
+In the sample, N is 3 and the lines are `a` (length 1), `abc` (length 3), and `ab` (length 2). The longest is `abc` with length 3, so the program prints `3`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- N is a valid whole number matching the number of lines that follow.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3788,16 +3794,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Path Extension. Read the input values and print the required result exactly.
+          <t>A media library organizes uploaded files by type using the text after the last dot in the file name, but some files are uploaded with no dot at all and need special handling.
+Write a program that reads a file name and prints the text after the last `.` in the name (without the dot itself). If the name has no dot, print `none`.
 ### Input Format
-- Line 1: Path
+- Line 1: A file name
 ### Output Format
 ```
 txt
 ```
+### Example Walkthrough
+In the sample, the file name is `a.txt`. The text after the last dot is `txt`, so the program prints `txt`. A name with no dot, like `README`, would print `none`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input is a valid file name with no spaces.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3941,16 +3950,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for CSV Column Count. Read the input values and print the required result exactly.
+          <t>A CSV import validator checks how many columns each row of a spreadsheet export has, to make sure every row matches the expected column count before the data is processed further.
+Write a program that reads one line representing a CSV row (values separated by commas) and prints how many columns it has. If the line is empty, print `0`.
 ### Input Format
-- Line 1: CSV row
+- Line 1: A CSV row (comma-separated values)
 ### Output Format
 ```
 3
 ```
+### Example Walkthrough
+In the sample, the row is `a,b,c`. Splitting on commas gives three values, so the program prints `3`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input is a single valid line representing one CSV row.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5500,17 +5512,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for JSON Key Value. Read the input values and print the required result exactly.
+          <t>A config loader reads a single JSON object representing an app's settings and needs to fetch one setting by name, reporting `Missing` if that setting isn't present in the file.
+Write a program that reads a line of JSON representing an object, parses it, reads a key on the next line, and prints the value for that key if it exists, or `Missing` otherwise.
 ### Input Format
-- Line 1: JSON object
-- Line 2: Key
+- Line 1: A JSON object
+- Line 2: The key to look up
 ### Output Format
 ```
 Asha
 ```
+### Example Walkthrough
+In the sample, the JSON is `{"name":"Asha","age":19}` and the key is `name`. Looking up `name` in the parsed object gives `Asha`, so the program prints `Asha`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input is valid JSON representing an object.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -5662,17 +5677,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Glob Suffix Match. Read the input values and print the required result exactly.
+          <t>A backup tool scans a folder's file list to count how many files match a certain extension pattern (like a simplified `*.py` glob), to decide whether a backup step is needed for that file type.
+Write a program that reads a line of space-separated file names, reads a suffix on the next line, and prints how many of the file names end with that exact suffix.
 ### Input Format
-- Line 1: File names
-- Line 2: Suffix
+- Line 1: Space-separated file names
+- Line 2: A suffix (e.g. `.py`)
 ### Output Format
 ```
 2
 ```
+### Example Walkthrough
+In the sample, the file names are `a.py b.txt c.py` and the suffix is `.py`. Two of the three file names (`a.py` and `c.py`) end with `.py`, so the program prints `2`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The inputs are valid, non-empty lines of text.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -5823,17 +5841,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Context Summary. Read the input values and print the required result exactly.
+          <t>A document analytics tool reads through a file's contents (opened safely with a `with` statement so it always closes properly) and needs to report the total number of characters across all its lines, not counting the line breaks between them.
+Write a program that reads a whole number N, then reads N more lines (treat them as the file's contents), and prints the total number of characters across all N lines combined. If N is 0, print `0`.
 ### Input Format
-- Line 1: N
-- Next N lines: Text
+- Line 1: N, the number of lines in the file
+- Next N lines: the file's contents
 ### Output Format
 ```
 4
 ```
+### Example Walkthrough
+In the sample, N is 2 and the lines are `ab` (2 characters) and `cd` (2 characters). Adding their lengths gives 2 + 2 = 4, so the program prints `4`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- N is a valid whole number matching the number of lines that follow.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7371,17 +7392,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for CSV Sum Column. Read the input values and print the required result exactly.
+          <t>An accounting import tool reads N rows of a CSV export where each row has an item label and an amount separated by a comma, and needs the total of just the amount column across all rows.
+Write a program that reads a whole number N, then reads N more lines each in the form `label,amount`, and prints the sum of the amount values. If N is 0, print `0`.
 ### Input Format
-- Line 1: N
-- Next N lines: name,value
+- Line 1: N, the number of rows
+- Next N lines: `label,amount`
 ### Output Format
 ```
 30
 ```
+### Example Walkthrough
+In the sample, N is 2 with rows `a,10` and `b,20`. Adding the amounts gives 10 + 20 = 30, so the program prints `30`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- N is a valid whole number, and every amount is a valid whole number.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7540,16 +7564,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for JSON List Average. Read the input values and print the required result exactly.
+          <t>A fitness app stores a week's daily step counts as a JSON array in a log file and needs the average steps per day to show on the weekly summary screen.
+Write a program that reads a line containing a JSON array of numbers, parses it, and prints the average of the numbers (their sum divided by how many there are).
 ### Input Format
-- Line 1: JSON list
+- Line 1: A JSON array of numbers
 ### Output Format
 ```
 2.0
 ```
+### Example Walkthrough
+In the sample, the array is `[1,2,3]`. The average is (1 + 2 + 3) / 3 = 2.0, so the program prints `2.0`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input is a valid, non-empty JSON array of numbers.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -7694,17 +7721,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Missing File Guard. Read the input values and print the required result exactly.
+          <t>A file cleanup script checks a requested file name against the set of files that actually exist in a folder before attempting to open or delete it, to avoid a crash from trying to act on a file that isn't there.
+Write a program that reads a line of space-separated file names (the files that exist), reads one more file name on the next line, and prints `Found` if that file name is in the list, or `Missing` otherwise.
 ### Input Format
-- Line 1: Available names
-- Line 2: Requested name
+- Line 1: Space-separated file names (the files that exist)
+- Line 2: The file name being requested
 ### Output Format
 ```
 Found
 ```
+### Example Walkthrough
+In the sample, the existing files are `a.txt b.txt` and the requested file is `a.txt`. Since `a.txt` is in the list, the program prints `Found`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The inputs are valid, non-empty lines of text.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>